<commit_message>
Snapshots re-fetched 2026-09-15 after the raw data loss; fixtures frozen on the new set, 2026-09-12 files kept
</commit_message>
<xml_diff>
--- a/data/out/capability_table.xlsx
+++ b/data/out/capability_table.xlsx
@@ -1158,12 +1158,12 @@
       </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY2" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY3" t="inlineStr">
@@ -2164,12 +2164,12 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY4" t="inlineStr">
@@ -2591,12 +2591,12 @@
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY5" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY6" t="inlineStr">
@@ -3525,12 +3525,12 @@
       </c>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX7" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY7" t="inlineStr">
@@ -3976,12 +3976,12 @@
       </c>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX8" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY8" t="inlineStr">
@@ -4427,12 +4427,12 @@
       </c>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX9" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY9" t="inlineStr">
@@ -4926,12 +4926,12 @@
       </c>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX10" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY10" t="inlineStr">
@@ -5425,12 +5425,12 @@
       </c>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX11" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY11" t="inlineStr">
@@ -5864,12 +5864,12 @@
       </c>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX12" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY12" t="inlineStr">
@@ -6259,12 +6259,12 @@
       </c>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX13" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY13" t="inlineStr">
@@ -6710,12 +6710,12 @@
       </c>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX14" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY14" t="inlineStr">
@@ -7217,12 +7217,12 @@
       </c>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX15" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY15" t="inlineStr">
@@ -7716,12 +7716,12 @@
       </c>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX16" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY16" t="inlineStr">
@@ -8167,12 +8167,12 @@
       </c>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX17" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY17" t="inlineStr">
@@ -8666,12 +8666,12 @@
       </c>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX18" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY18" t="inlineStr">
@@ -9169,12 +9169,12 @@
       </c>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX19" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY19" t="inlineStr">
@@ -9672,12 +9672,12 @@
       </c>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY20" t="inlineStr">
@@ -10127,12 +10127,12 @@
       </c>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX21" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY21" t="inlineStr">
@@ -10618,12 +10618,12 @@
       </c>
       <c r="AW22" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX22" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY22" t="inlineStr">
@@ -11109,12 +11109,12 @@
       </c>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX23" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY23" t="inlineStr">
@@ -11564,12 +11564,12 @@
       </c>
       <c r="AW24" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX24" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY24" t="inlineStr">
@@ -12023,12 +12023,12 @@
       </c>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX25" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY25" t="inlineStr">
@@ -12522,12 +12522,12 @@
       </c>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX26" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY26" t="inlineStr">
@@ -13021,12 +13021,12 @@
       </c>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX27" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY27" t="inlineStr">
@@ -13464,12 +13464,12 @@
       </c>
       <c r="AW28" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX28" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY28" t="inlineStr">
@@ -13915,12 +13915,12 @@
       </c>
       <c r="AW29" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX29" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY29" t="inlineStr">
@@ -14358,12 +14358,12 @@
       </c>
       <c r="AW30" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX30" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY30" t="inlineStr">
@@ -14857,12 +14857,12 @@
       </c>
       <c r="AW31" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX31" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY31" t="inlineStr">
@@ -15356,12 +15356,12 @@
       </c>
       <c r="AW32" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX32" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY32" t="inlineStr">
@@ -15839,12 +15839,12 @@
       </c>
       <c r="AW33" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX33" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY33" t="inlineStr">
@@ -16290,12 +16290,12 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX34" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY34" t="inlineStr">
@@ -16705,12 +16705,12 @@
       </c>
       <c r="AW35" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX35" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY35" t="inlineStr">
@@ -17148,12 +17148,12 @@
       </c>
       <c r="AW36" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX36" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY36" t="inlineStr">
@@ -17551,12 +17551,12 @@
       </c>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX37" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY37" t="inlineStr">
@@ -17998,12 +17998,12 @@
       </c>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX38" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY38" t="inlineStr">
@@ -18453,12 +18453,12 @@
       </c>
       <c r="AW39" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX39" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY39" t="inlineStr">
@@ -18936,12 +18936,12 @@
       </c>
       <c r="AW40" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX40" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY40" t="inlineStr">
@@ -19387,12 +19387,12 @@
       </c>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX41" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY41" t="inlineStr">
@@ -19822,12 +19822,12 @@
       </c>
       <c r="AW42" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX42" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY42" t="inlineStr">
@@ -20281,12 +20281,12 @@
       </c>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX43" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY43" t="inlineStr">
@@ -20784,12 +20784,12 @@
       </c>
       <c r="AW44" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX44" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY44" t="inlineStr">
@@ -21243,12 +21243,12 @@
       </c>
       <c r="AW45" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX45" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY45" t="inlineStr">
@@ -21706,12 +21706,12 @@
       </c>
       <c r="AW46" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX46" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY46" t="inlineStr">
@@ -22205,12 +22205,12 @@
       </c>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX47" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY47" t="inlineStr">
@@ -22712,12 +22712,12 @@
       </c>
       <c r="AW48" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX48" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY48" t="inlineStr">
@@ -23219,12 +23219,12 @@
       </c>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX49" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY49" t="inlineStr">
@@ -23726,12 +23726,12 @@
       </c>
       <c r="AW50" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX50" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY50" t="inlineStr">
@@ -24229,12 +24229,12 @@
       </c>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX51" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY51" t="inlineStr">
@@ -24740,12 +24740,12 @@
       </c>
       <c r="AW52" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX52" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY52" t="inlineStr">
@@ -25251,12 +25251,12 @@
       </c>
       <c r="AW53" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX53" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY53" t="inlineStr">
@@ -25754,12 +25754,12 @@
       </c>
       <c r="AW54" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX54" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY54" t="inlineStr">
@@ -26205,12 +26205,12 @@
       </c>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX55" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY55" t="inlineStr">
@@ -26541,7 +26541,7 @@
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>In the vicinity of the Library (Lot 348). 7am-5pm daily.</t>
+          <t>In the vicinity of the Library (Lot 348). 7am-5pm daily. Free WiFi is on the way for Angurugu: Free community Wi-Fi on the way - Angurugu</t>
         </is>
       </c>
       <c r="W56" t="inlineStr">
@@ -26593,7 +26593,7 @@
       </c>
       <c r="AH56" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="AI56" t="inlineStr">
@@ -26660,12 +26660,12 @@
       </c>
       <c r="AW56" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX56" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY56" t="inlineStr">
@@ -27127,12 +27127,12 @@
       </c>
       <c r="AW57" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX57" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY57" t="inlineStr">
@@ -27530,12 +27530,12 @@
       </c>
       <c r="AW58" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX58" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY58" t="inlineStr">
@@ -27941,12 +27941,12 @@
       </c>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX59" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY59" t="inlineStr">
@@ -28348,12 +28348,12 @@
       </c>
       <c r="AW60" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX60" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY60" t="inlineStr">
@@ -28811,12 +28811,12 @@
       </c>
       <c r="AW61" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX61" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY61" t="inlineStr">
@@ -29266,12 +29266,12 @@
       </c>
       <c r="AW62" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX62" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY62" t="inlineStr">
@@ -29717,12 +29717,12 @@
       </c>
       <c r="AW63" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX63" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY63" t="inlineStr">
@@ -30212,12 +30212,12 @@
       </c>
       <c r="AW64" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX64" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY64" t="inlineStr">
@@ -30651,12 +30651,12 @@
       </c>
       <c r="AW65" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX65" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY65" t="inlineStr">
@@ -31054,12 +31054,12 @@
       </c>
       <c r="AW66" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX66" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY66" t="inlineStr">
@@ -31385,12 +31385,12 @@
       </c>
       <c r="U67" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="V67" t="inlineStr">
         <is>
-          <t>In the vicinity of the Lot 184, Gadapu Rd. 8am-8pm daily.</t>
+          <t>There is free wifi at the Rulku Lodge for guests. Milingimbi is included in the Federal and Northern Territory Government funding package for the roll out of free Wifi in remote NT communities . Telstra has 3G and 4G coverage on the island.</t>
         </is>
       </c>
       <c r="W67" t="inlineStr">
@@ -31442,7 +31442,7 @@
       </c>
       <c r="AH67" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="AI67" t="inlineStr">
@@ -31509,12 +31509,12 @@
       </c>
       <c r="AW67" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX67" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY67" t="inlineStr">
@@ -32004,12 +32004,12 @@
       </c>
       <c r="AW68" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX68" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY68" t="inlineStr">
@@ -32411,12 +32411,12 @@
       </c>
       <c r="AW69" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX69" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY69" t="inlineStr">
@@ -32902,12 +32902,12 @@
       </c>
       <c r="AW70" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX70" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY70" t="inlineStr">
@@ -33409,12 +33409,12 @@
       </c>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX71" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY71" t="inlineStr">
@@ -33912,12 +33912,12 @@
       </c>
       <c r="AW72" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX72" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY72" t="inlineStr">
@@ -34359,12 +34359,12 @@
       </c>
       <c r="AW73" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX73" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY73" t="inlineStr">
@@ -34846,12 +34846,12 @@
       </c>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX74" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY74" t="inlineStr">
@@ -35349,12 +35349,12 @@
       </c>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX75" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY75" t="inlineStr">
@@ -35848,12 +35848,12 @@
       </c>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX76" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY76" t="inlineStr">
@@ -36339,12 +36339,12 @@
       </c>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AX77" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY77" t="inlineStr">
@@ -36822,12 +36822,12 @@
       </c>
       <c r="AW78" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX78" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY78" t="inlineStr">
@@ -37305,12 +37305,12 @@
       </c>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX79" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY79" t="inlineStr">
@@ -37804,12 +37804,12 @@
       </c>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX80" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY80" t="inlineStr">
@@ -38295,12 +38295,12 @@
       </c>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX81" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY81" t="inlineStr">
@@ -38774,12 +38774,12 @@
       </c>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX82" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY82" t="inlineStr">
@@ -39221,12 +39221,12 @@
       </c>
       <c r="AW83" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY83" t="inlineStr">
@@ -39680,12 +39680,12 @@
       </c>
       <c r="AW84" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX84" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY84" t="inlineStr">
@@ -40171,12 +40171,12 @@
       </c>
       <c r="AW85" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX85" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY85" t="inlineStr">
@@ -40658,12 +40658,12 @@
       </c>
       <c r="AW86" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX86" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY86" t="inlineStr">
@@ -41149,12 +41149,12 @@
       </c>
       <c r="AW87" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX87" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY87" t="inlineStr">
@@ -41600,12 +41600,12 @@
       </c>
       <c r="AW88" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX88" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY88" t="inlineStr">
@@ -42111,12 +42111,12 @@
       </c>
       <c r="AW89" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX89" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY89" t="inlineStr">
@@ -42602,12 +42602,12 @@
       </c>
       <c r="AW90" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX90" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY90" t="inlineStr">
@@ -43053,12 +43053,12 @@
       </c>
       <c r="AW91" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX91" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY91" t="inlineStr">
@@ -43464,12 +43464,12 @@
       </c>
       <c r="AW92" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AX92" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY92" t="inlineStr">
@@ -43939,12 +43939,12 @@
       </c>
       <c r="AW93" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX93" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY93" t="inlineStr">
@@ -44427,12 +44427,12 @@
       </c>
       <c r="AW94" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX94" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY94" t="inlineStr">
@@ -44874,12 +44874,12 @@
       </c>
       <c r="AW95" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX95" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY95" t="inlineStr">
@@ -45281,12 +45281,12 @@
       </c>
       <c r="AW96" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX96" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY96" t="inlineStr">
@@ -45676,12 +45676,12 @@
       </c>
       <c r="AW97" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AX97" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AY97" t="inlineStr">

</xml_diff>

<commit_message>
Task-39 DONE: map-claim reliability model on the Audit, AUC 0.79, ships as one word per community
</commit_message>
<xml_diff>
--- a/data/out/capability_table.xlsx
+++ b/data/out/capability_table.xlsx
@@ -1301,7 +1301,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW2" t="inlineStr"/>
       <c r="BX2" t="inlineStr"/>
       <c r="BY2" t="inlineStr"/>
@@ -4598,7 +4602,11 @@
           <t>Within 100 metres</t>
         </is>
       </c>
-      <c r="BV9" t="inlineStr"/>
+      <c r="BV9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW9" t="inlineStr"/>
       <c r="BX9" t="inlineStr"/>
       <c r="BY9" t="inlineStr"/>
@@ -5101,7 +5109,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV10" t="inlineStr"/>
+      <c r="BV10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW10" t="inlineStr">
         <is>
           <t>11.2</t>
@@ -6462,7 +6474,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV13" t="inlineStr"/>
+      <c r="BV13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW13" t="inlineStr">
         <is>
           <t>31.4</t>
@@ -6925,7 +6941,11 @@
           <t>Within 100 metres</t>
         </is>
       </c>
-      <c r="BV14" t="inlineStr"/>
+      <c r="BV14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW14" t="inlineStr"/>
       <c r="BX14" t="inlineStr"/>
       <c r="BY14" t="inlineStr"/>
@@ -10865,7 +10885,11 @@
           <t>Within 100 metres</t>
         </is>
       </c>
-      <c r="BV22" t="inlineStr"/>
+      <c r="BV22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW22" t="inlineStr"/>
       <c r="BX22" t="inlineStr"/>
       <c r="BY22" t="inlineStr"/>
@@ -11360,7 +11384,11 @@
           <t>Within 100 metres</t>
         </is>
       </c>
-      <c r="BV23" t="inlineStr"/>
+      <c r="BV23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW23" t="inlineStr"/>
       <c r="BX23" t="inlineStr"/>
       <c r="BY23" t="inlineStr"/>
@@ -11819,7 +11847,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV24" t="inlineStr"/>
+      <c r="BV24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW24" t="inlineStr"/>
       <c r="BX24" t="inlineStr"/>
       <c r="BY24" t="inlineStr"/>
@@ -13743,7 +13775,11 @@
           <t>Within 100 metres</t>
         </is>
       </c>
-      <c r="BV28" t="inlineStr"/>
+      <c r="BV28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW28" t="inlineStr"/>
       <c r="BX28" t="inlineStr"/>
       <c r="BY28" t="inlineStr"/>
@@ -14653,7 +14689,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="BV30" t="inlineStr"/>
+      <c r="BV30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW30" t="inlineStr">
         <is>
           <t>16.8</t>
@@ -15164,7 +15204,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV31" t="inlineStr"/>
+      <c r="BV31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW31" t="inlineStr">
         <is>
           <t>23.6</t>
@@ -15675,7 +15719,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV32" t="inlineStr"/>
+      <c r="BV32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW32" t="inlineStr"/>
       <c r="BX32" t="inlineStr"/>
       <c r="BY32" t="inlineStr"/>
@@ -17036,7 +17084,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV35" t="inlineStr"/>
+      <c r="BV35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW35" t="inlineStr">
         <is>
           <t>21.2</t>
@@ -17898,7 +17950,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV37" t="inlineStr"/>
+      <c r="BV37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW37" t="inlineStr"/>
       <c r="BX37" t="inlineStr"/>
       <c r="BY37" t="inlineStr"/>
@@ -18349,7 +18405,11 @@
           <t>Within 100 metres</t>
         </is>
       </c>
-      <c r="BV38" t="inlineStr"/>
+      <c r="BV38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW38" t="inlineStr"/>
       <c r="BX38" t="inlineStr"/>
       <c r="BY38" t="inlineStr"/>
@@ -19750,7 +19810,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV41" t="inlineStr"/>
+      <c r="BV41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW41" t="inlineStr"/>
       <c r="BX41" t="inlineStr"/>
       <c r="BY41" t="inlineStr"/>
@@ -20652,7 +20716,11 @@
           <t>Within 100 metres</t>
         </is>
       </c>
-      <c r="BV43" t="inlineStr"/>
+      <c r="BV43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW43" t="inlineStr"/>
       <c r="BX43" t="inlineStr"/>
       <c r="BY43" t="inlineStr"/>
@@ -21159,7 +21227,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="BV44" t="inlineStr"/>
+      <c r="BV44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW44" t="inlineStr"/>
       <c r="BX44" t="inlineStr"/>
       <c r="BY44" t="inlineStr"/>
@@ -23630,7 +23702,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="BV49" t="inlineStr"/>
+      <c r="BV49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW49" t="inlineStr"/>
       <c r="BX49" t="inlineStr"/>
       <c r="BY49" t="inlineStr"/>
@@ -24141,7 +24217,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV50" t="inlineStr"/>
+      <c r="BV50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW50" t="inlineStr"/>
       <c r="BX50" t="inlineStr"/>
       <c r="BY50" t="inlineStr"/>
@@ -24648,7 +24728,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV51" t="inlineStr"/>
+      <c r="BV51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW51" t="inlineStr"/>
       <c r="BX51" t="inlineStr"/>
       <c r="BY51" t="inlineStr"/>
@@ -25678,7 +25762,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="BV53" t="inlineStr"/>
+      <c r="BV53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW53" t="inlineStr"/>
       <c r="BX53" t="inlineStr"/>
       <c r="BY53" t="inlineStr"/>
@@ -26640,7 +26728,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV55" t="inlineStr"/>
+      <c r="BV55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW55" t="inlineStr"/>
       <c r="BX55" t="inlineStr"/>
       <c r="BY55" t="inlineStr"/>
@@ -33421,7 +33513,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="BV70" t="inlineStr"/>
+      <c r="BV70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW70" t="inlineStr"/>
       <c r="BX70" t="inlineStr"/>
       <c r="BY70" t="inlineStr"/>
@@ -35381,7 +35477,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="BV74" t="inlineStr"/>
+      <c r="BV74" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW74" t="inlineStr">
         <is>
           <t>21.1</t>
@@ -36415,7 +36515,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV76" t="inlineStr"/>
+      <c r="BV76" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW76" t="inlineStr">
         <is>
           <t>15.6</t>
@@ -36918,7 +37022,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV77" t="inlineStr"/>
+      <c r="BV77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW77" t="inlineStr">
         <is>
           <t>14.9</t>
@@ -37413,7 +37521,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV78" t="inlineStr"/>
+      <c r="BV78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW78" t="inlineStr">
         <is>
           <t>18.7</t>
@@ -37908,7 +38020,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV79" t="inlineStr"/>
+      <c r="BV79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW79" t="inlineStr"/>
       <c r="BX79" t="inlineStr"/>
       <c r="BY79" t="inlineStr"/>
@@ -40335,7 +40451,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="BV84" t="inlineStr"/>
+      <c r="BV84" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW84" t="inlineStr">
         <is>
           <t>18.9</t>
@@ -40838,7 +40958,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV85" t="inlineStr"/>
+      <c r="BV85" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW85" t="inlineStr">
         <is>
           <t>12.3</t>
@@ -42802,7 +42926,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="BV89" t="inlineStr"/>
+      <c r="BV89" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW89" t="inlineStr"/>
       <c r="BX89" t="inlineStr"/>
       <c r="BY89" t="inlineStr"/>
@@ -43752,7 +43880,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV91" t="inlineStr"/>
+      <c r="BV91" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW91" t="inlineStr"/>
       <c r="BX91" t="inlineStr"/>
       <c r="BY91" t="inlineStr"/>
@@ -44167,7 +44299,11 @@
           <t>Within 100 metres</t>
         </is>
       </c>
-      <c r="BV92" t="inlineStr"/>
+      <c r="BV92" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW92" t="inlineStr">
         <is>
           <t>11.4</t>
@@ -44654,7 +44790,11 @@
           <t>Within 10 metres</t>
         </is>
       </c>
-      <c r="BV93" t="inlineStr"/>
+      <c r="BV93" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW93" t="inlineStr"/>
       <c r="BX93" t="inlineStr"/>
       <c r="BY93" t="inlineStr"/>
@@ -45605,7 +45745,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="BV95" t="inlineStr"/>
+      <c r="BV95" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW95" t="inlineStr">
         <is>
           <t>36.2</t>
@@ -46423,7 +46567,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="BV97" t="inlineStr"/>
+      <c r="BV97" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="BW97" t="inlineStr"/>
       <c r="BX97" t="inlineStr"/>
       <c r="BY97" t="inlineStr"/>

</xml_diff>